<commit_message>
Tot stap 4 gemaakt
</commit_message>
<xml_diff>
--- a/DE samenwerken/Week 6/Logboek.xlsx
+++ b/DE samenwerken/Week 6/Logboek.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gebruiker\source\repos\DEAI_portfolio\DE samenwerken\Week 6\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6561DCD5-7CFC-4753-AAFA-39801756D92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="12000" yWindow="0" windowWidth="12000" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,25 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>Features</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>SalePrice</t>
+  </si>
+  <si>
+    <t>Gr Liv Area, Overall Qual, Neighborhood</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -53,7 +76,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -330,10 +353,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="37.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Opmaak logboek aan ge past
</commit_message>
<xml_diff>
--- a/DE samenwerken/Week 6/Logboek.xlsx
+++ b/DE samenwerken/Week 6/Logboek.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gebruiker\source\repos\DEAI_portfolio\DE samenwerken\Week 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1338497A-1DE8-4AB3-90A5-4EE481C04D46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F9A25DF-3410-4EA4-812F-031E3096016C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12000" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Features</t>
   </si>
@@ -36,19 +36,31 @@
     <t>SalePrice</t>
   </si>
   <si>
-    <t>Gr Liv Area, Overall Qual, Neighborhood</t>
-  </si>
-  <si>
     <t>Hyperparamaters</t>
   </si>
   <si>
-    <t>fit_intercept=True, positive=False</t>
-  </si>
-  <si>
     <t>Resultaten</t>
   </si>
   <si>
-    <t>MSE: 1525093881.3938231, R2: 0.8097805096350512</t>
+    <t>R2: 0.8097805096350512</t>
+  </si>
+  <si>
+    <t>MSE: 1525093881.3938231</t>
+  </si>
+  <si>
+    <t>fit_intercept=True</t>
+  </si>
+  <si>
+    <t>positive=False</t>
+  </si>
+  <si>
+    <t>Gr Liv Area</t>
+  </si>
+  <si>
+    <t>Overall Qual</t>
+  </si>
+  <si>
+    <t>Neighborhood</t>
   </si>
 </sst>
 </file>
@@ -101,6 +113,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CC9D797F-4CED-4B4A-B6E9-41FB7C35005D}" name="Tabel1" displayName="Tabel1" ref="A1:D4" totalsRowShown="0">
+  <autoFilter ref="A1:D4" xr:uid="{CC9D797F-4CED-4B4A-B6E9-41FB7C35005D}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{0904ECDB-157B-4BDD-BB62-014B67DA9584}" name="Target"/>
+    <tableColumn id="2" xr3:uid="{567C2AB2-970A-40C9-B710-732F559D5C69}" name="Features"/>
+    <tableColumn id="3" xr3:uid="{4BAC2826-D838-40B2-AA58-BFDA5E3D29EB}" name="Hyperparamaters"/>
+    <tableColumn id="4" xr3:uid="{66B9318C-2084-4A10-8CE7-ADE5D922275B}" name="Resultaten"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -366,46 +391,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="46.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>